<commit_message>
plants_abroad: Fix irrefuehrende "Dreieck"-Notiz bei Drittland-Ausfuhr (GB)
Die Herleitungs-Notiz setzte "(Dreieck)" pauschal, sobald der Warenempfaenger
keine EPDE/EPROHA-UID hat — auch bei Nicht-EU-Zielen. Ein Dreiecksgeschaeft
(Art. 141) setzt aber DREI EU-Mitgliedstaaten voraus; GB (Drittland) ist eine
Ausfuhr, kein Dreieck.

- Notiz nur noch "(Dreieck, Art. 141)" wenn Ship-to in der EU liegt; sonst
  "Drittland-Ausfuhr ueber Heimat-UID; KEIN Dreieck"
- Betroffen: EPDE "Strecke DE/EU -> WE GB", EPROHA "Ausfuhr AT -> GB"
- Kennzeichen (G0/A0/D0) und Treatment (Ausfuhr) waren bereits korrekt —
  nur die Notiz war irrefuehrend
- 8 Original-Zeilen werden weiterhin exakt reproduziert

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BMKbRkyEepa3uat53j1you
</commit_message>
<xml_diff>
--- a/vat-knowledge/plants_abroad/Matrix_erweitert_EPDE.xlsx
+++ b/vat-knowledge/plants_abroad/Matrix_erweitert_EPDE.xlsx
@@ -602,68 +602,68 @@
           <t>Lagerauftrag Werk PL – WE Polen (Inland)</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>1702</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>PL5263841834</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="J2" s="9" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>PLxxx</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="M2" s="9" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N2" s="9" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O2" s="9" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -676,68 +676,68 @@
           <t>Lagerauftrag Werk PL – WE Italien (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>1702</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>PL5263841834</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N3" s="9" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -750,68 +750,68 @@
           <t>Lagerauftrag Werk PL – WE Deutschland (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>1702</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>PL5263841834</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L4" s="10" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N4" s="9" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -824,68 +824,68 @@
           <t>Lagerauftrag Werk PL – WE Tschechien (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>1702</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>PL5263841834</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>CZxxx</t>
         </is>
       </c>
-      <c r="L5" s="10" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="M5" s="9" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N5" s="9" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O5" s="9" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -898,68 +898,68 @@
           <t>Lagerauftrag Werk CZ – WE Tschechien (Inland)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>1703</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>CZ687387072</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="K6" s="9" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>CZxxx</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>AE</t>
         </is>
       </c>
-      <c r="M6" s="9" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N6" s="9" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O6" s="9" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -972,68 +972,68 @@
           <t>Lagerauftrag Werk CZ – WE Slowakei (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>1703</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>CZ687387072</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>SK</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>SKxxx</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>OB</t>
         </is>
       </c>
-      <c r="M7" s="9" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1046,68 +1046,68 @@
           <t>Lagerauftrag Werk CZ – WE Deutschland (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>1703</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>CZ687387072</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="K8" s="9" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L8" s="10" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>OB</t>
         </is>
       </c>
-      <c r="M8" s="9" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N8" s="9" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O8" s="9" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1120,68 +1120,68 @@
           <t>Lagerauftrag Werk DE – WE Deutschland (Inland)</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J9" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="K9" s="9" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L9" s="10" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>DS</t>
         </is>
       </c>
-      <c r="M9" s="9" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N9" s="9" t="inlineStr">
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O9" s="9" t="inlineStr">
+      <c r="O9" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1194,68 +1194,68 @@
           <t>Lagerauftrag Werk DE – WE Frankreich (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I10" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J10" s="9" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="K10" s="9" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>FRxxx</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M10" s="9" t="inlineStr">
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N10" s="9" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O10" s="9" t="inlineStr">
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1268,68 +1268,68 @@
           <t>Strecke – Lieferant DE/EU (≠PL) – WE Polen</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>PL5263841834</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="J11" s="9" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="K11" s="9" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>PLxxx</t>
         </is>
       </c>
-      <c r="L11" s="10" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="M11" s="9" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N11" s="9" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O11" s="9" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1342,68 +1342,68 @@
           <t>Strecke – Lieferant DE/EU (≠CZ) – WE Tschechien</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>CZ687387072</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="J12" s="9" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="K12" s="9" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>CZxxx</t>
         </is>
       </c>
-      <c r="L12" s="10" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>AE</t>
         </is>
       </c>
-      <c r="M12" s="9" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N12" s="9" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O12" s="9" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1416,68 +1416,68 @@
           <t>Strecke – Lieferant DE/EU (≠SI) – WE Slowenien</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>SI66423562</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I13" s="9" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="J13" s="9" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>SIxxx</t>
         </is>
       </c>
-      <c r="L13" s="10" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>CB</t>
         </is>
       </c>
-      <c r="M13" s="9" t="inlineStr">
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N13" s="9" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O13" s="9" t="inlineStr">
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1490,68 +1490,68 @@
           <t>Strecke – Lieferant Schweden – WE Slowenien</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
           <t>SI66423562</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>SE</t>
         </is>
       </c>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="J14" s="9" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K14" s="9" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>SIxxx</t>
         </is>
       </c>
-      <c r="L14" s="10" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>CB</t>
         </is>
       </c>
-      <c r="M14" s="9" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N14" s="9" t="inlineStr">
+      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O14" s="9" t="inlineStr">
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1564,68 +1564,68 @@
           <t>Strecke – Lieferant DE/EU (≠BE) – WE Belgien</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>BE1022245089</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="J15" s="9" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>BExxx</t>
         </is>
       </c>
-      <c r="L15" s="10" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>BS</t>
         </is>
       </c>
-      <c r="M15" s="9" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N15" s="9" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
+      <c r="O15" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1638,48 +1638,48 @@
           <t>Strecke – Lieferant DE/EU (≠NL) – WE Niederlande</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>NL827914052B01</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I16" s="9" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>NL</t>
         </is>
       </c>
-      <c r="J16" s="9" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>NL</t>
         </is>
       </c>
-      <c r="K16" s="9" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>NLxxx</t>
         </is>
@@ -1689,17 +1689,17 @@
           <t>⚠ kein SAP-Stkz (Lücke)</t>
         </is>
       </c>
-      <c r="M16" s="9" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N16" s="9" t="inlineStr">
+      <c r="N16" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O16" s="9" t="inlineStr">
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1712,68 +1712,68 @@
           <t>Strecke – Lieferant DE/EU (≠LV) – WE Lettland</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
           <t>LV90013367396</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>LV</t>
         </is>
       </c>
-      <c r="J17" s="9" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>LV</t>
         </is>
       </c>
-      <c r="K17" s="9" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>LVxxx</t>
         </is>
       </c>
-      <c r="L17" s="10" t="inlineStr">
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>LS</t>
         </is>
       </c>
-      <c r="M17" s="9" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N17" s="9" t="inlineStr">
+      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O17" s="9" t="inlineStr">
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1786,68 +1786,68 @@
           <t>Strecke – Lieferant DE/EU (≠EE) – WE Estland</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
           <t>EE102839441</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I18" s="9" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>EE</t>
         </is>
       </c>
-      <c r="J18" s="9" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>EE</t>
         </is>
       </c>
-      <c r="K18" s="9" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>EExxx</t>
         </is>
       </c>
-      <c r="L18" s="10" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="M18" s="9" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N18" s="9" t="inlineStr">
+      <c r="N18" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O18" s="9" t="inlineStr">
+      <c r="O18" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1860,75 +1860,75 @@
           <t>Strecke – Lieferant Slowenien – WE Ungarn (Dreieck)</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="I19" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J19" s="9" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="K19" s="9" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>HUxxx</t>
         </is>
       </c>
-      <c r="L19" s="10" t="inlineStr">
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M19" s="9" t="inlineStr">
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N19" s="9" t="inlineStr">
+      <c r="N19" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O19" s="9" t="inlineStr">
+      <c r="O19" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck)</t>
+          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck, Art. 141)</t>
         </is>
       </c>
     </row>
@@ -1938,75 +1938,75 @@
           <t>Strecke – Lieferant Italien – WE Frankreich (Dreieck)</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="I20" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J20" s="9" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="K20" s="9" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>FRxxx</t>
         </is>
       </c>
-      <c r="L20" s="10" t="inlineStr">
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M20" s="9" t="inlineStr">
+      <c r="M20" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N20" s="9" t="inlineStr">
+      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O20" s="9" t="inlineStr">
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck)</t>
+          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck, Art. 141)</t>
         </is>
       </c>
     </row>
@@ -2016,75 +2016,75 @@
           <t>Strecke – Lieferant Polen – WE Spanien (Dreieck)</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I21" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J21" s="9" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="K21" s="9" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>ESxxx</t>
         </is>
       </c>
-      <c r="L21" s="10" t="inlineStr">
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M21" s="9" t="inlineStr">
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N21" s="9" t="inlineStr">
+      <c r="N21" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O21" s="9" t="inlineStr">
+      <c r="O21" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck)</t>
+          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck, Art. 141)</t>
         </is>
       </c>
     </row>
@@ -2094,75 +2094,75 @@
           <t>Strecke – Lieferant Frankreich – WE Österreich (Dreieck)</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J22" s="9" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>AT</t>
         </is>
       </c>
-      <c r="K22" s="9" t="inlineStr">
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>ATxxx</t>
         </is>
       </c>
-      <c r="L22" s="10" t="inlineStr">
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M22" s="9" t="inlineStr">
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N22" s="9" t="inlineStr">
+      <c r="N22" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O22" s="9" t="inlineStr">
+      <c r="O22" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck)</t>
+          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck, Art. 141)</t>
         </is>
       </c>
     </row>
@@ -2172,75 +2172,75 @@
           <t>Strecke – Lieferant Tschechien – WE Rumänien (Dreieck)</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J23" s="9" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>RO</t>
         </is>
       </c>
-      <c r="K23" s="9" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>ROxxx</t>
         </is>
       </c>
-      <c r="L23" s="10" t="inlineStr">
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M23" s="9" t="inlineStr">
+      <c r="M23" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N23" s="9" t="inlineStr">
+      <c r="N23" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O23" s="9" t="inlineStr">
+      <c r="O23" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck)</t>
+          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck, Art. 141)</t>
         </is>
       </c>
     </row>
@@ -2250,22 +2250,22 @@
           <t>Strecke EXW – Lieferant DE – WE Slowenien</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2275,47 +2275,47 @@
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H24" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I24" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J24" s="9" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K24" s="9" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>SIxxx</t>
         </is>
       </c>
-      <c r="L24" s="10" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M24" s="9" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N24" s="9" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O24" s="9" t="inlineStr">
+      <c r="O24" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2328,22 +2328,22 @@
           <t>Strecke EXW – Lieferant Slowenien (abgeholt) – WE Slowenien</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2353,47 +2353,47 @@
           <t>SI66423562</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H25" s="9" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="I25" s="9" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="J25" s="9" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K25" s="9" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>SIxxx</t>
         </is>
       </c>
-      <c r="L25" s="10" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>CB</t>
         </is>
       </c>
-      <c r="M25" s="9" t="inlineStr">
+      <c r="M25" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N25" s="9" t="inlineStr">
+      <c r="N25" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O25" s="9" t="inlineStr">
+      <c r="O25" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2406,22 +2406,22 @@
           <t>Strecke EXW – Lieferant Polen – WE Italien</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2431,47 +2431,47 @@
           <t>PL5263841834</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I26" s="9" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="J26" s="9" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K26" s="9" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L26" s="10" t="inlineStr">
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="M26" s="9" t="inlineStr">
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N26" s="9" t="inlineStr">
+      <c r="N26" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O26" s="9" t="inlineStr">
+      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2484,22 +2484,22 @@
           <t>Strecke EXW – Lieferant Tschechien – WE Deutschland</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2509,47 +2509,47 @@
           <t>CZ687387072</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H27" s="9" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="I27" s="9" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="J27" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="K27" s="9" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L27" s="10" t="inlineStr">
+      <c r="L27" s="4" t="inlineStr">
         <is>
           <t>OB</t>
         </is>
       </c>
-      <c r="M27" s="9" t="inlineStr">
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N27" s="9" t="inlineStr">
+      <c r="N27" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O27" s="9" t="inlineStr">
+      <c r="O27" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2562,22 +2562,22 @@
           <t>Strecke EXW – Lieferant Belgien – WE Belgien (Inland)</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2587,47 +2587,47 @@
           <t>BE1022245089</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H28" s="9" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="I28" s="9" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="J28" s="9" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="K28" s="9" t="inlineStr">
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>BExxx</t>
         </is>
       </c>
-      <c r="L28" s="10" t="inlineStr">
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>BS</t>
         </is>
       </c>
-      <c r="M28" s="9" t="inlineStr">
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>Inlandslieferung</t>
         </is>
       </c>
-      <c r="N28" s="9" t="inlineStr">
+      <c r="N28" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O28" s="9" t="inlineStr">
+      <c r="O28" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2640,22 +2640,22 @@
           <t>Strecke EXW – Lieferant Italien (ohne EPDE-UID) – WE Slowenien</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2665,47 +2665,47 @@
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H29" s="9" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="I29" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J29" s="9" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K29" s="9" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>SIxxx</t>
         </is>
       </c>
-      <c r="L29" s="10" t="inlineStr">
+      <c r="L29" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M29" s="9" t="inlineStr">
+      <c r="M29" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N29" s="9" t="inlineStr">
+      <c r="N29" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O29" s="9" t="inlineStr">
+      <c r="O29" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2722,22 +2722,22 @@
           <t>Strecke EXW – Lieferant Belgien – WE Frankreich (BE ig. Lief.)</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2747,27 +2747,27 @@
           <t>BE1022245089</t>
         </is>
       </c>
-      <c r="G30" s="9" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H30" s="9" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="I30" s="9" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="J30" s="9" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="K30" s="9" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>FRxxx</t>
         </is>
@@ -2777,17 +2777,17 @@
           <t>⚠ kein SAP-Stkz (Lücke)</t>
         </is>
       </c>
-      <c r="M30" s="9" t="inlineStr">
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N30" s="9" t="inlineStr">
+      <c r="N30" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O30" s="9" t="inlineStr">
+      <c r="O30" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2800,22 +2800,22 @@
           <t>Strecke EXW – Lieferant Niederlande – WE Deutschland (NL ig. Lief.)</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2825,27 +2825,27 @@
           <t>NL827914052B01</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H31" s="9" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>NL</t>
         </is>
       </c>
-      <c r="I31" s="9" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>NL</t>
         </is>
       </c>
-      <c r="J31" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="K31" s="9" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
@@ -2855,17 +2855,17 @@
           <t>⚠ kein SAP-Stkz (Lücke)</t>
         </is>
       </c>
-      <c r="M31" s="9" t="inlineStr">
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N31" s="9" t="inlineStr">
+      <c r="N31" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O31" s="9" t="inlineStr">
+      <c r="O31" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2878,48 +2878,48 @@
           <t>Lagerauftrag Werk PL – WE Schweiz (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>1702</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>PL5263841834</t>
         </is>
       </c>
-      <c r="G32" s="9" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H32" s="9" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I32" s="9" t="inlineStr">
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="J32" s="9" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K32" s="9" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
@@ -2929,17 +2929,17 @@
           <t>⚠ kein SAP-Stkz (Treatment fehlt: export)</t>
         </is>
       </c>
-      <c r="M32" s="9" t="inlineStr">
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>Ausfuhr</t>
         </is>
       </c>
-      <c r="N32" s="9" t="inlineStr">
+      <c r="N32" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O32" s="9" t="inlineStr">
+      <c r="O32" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -2952,68 +2952,68 @@
           <t>Lager DE – WE Schweiz (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr"/>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G33" s="9" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I33" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J33" s="9" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K33" s="9" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L33" s="10" t="inlineStr">
+      <c r="L33" s="4" t="inlineStr">
         <is>
           <t>G0</t>
         </is>
       </c>
-      <c r="M33" s="9" t="inlineStr">
+      <c r="M33" s="3" t="inlineStr">
         <is>
           <t>Ausfuhr</t>
         </is>
       </c>
-      <c r="N33" s="9" t="inlineStr">
+      <c r="N33" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O33" s="9" t="inlineStr">
+      <c r="O33" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -3026,68 +3026,68 @@
           <t>Lager DE – WE Liechtenstein (Ausfuhr, Schweizer MWST-Raum)</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr"/>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G34" s="9" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I34" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J34" s="9" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K34" s="9" t="inlineStr">
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L34" s="10" t="inlineStr">
+      <c r="L34" s="4" t="inlineStr">
         <is>
           <t>G0</t>
         </is>
       </c>
-      <c r="M34" s="9" t="inlineStr">
+      <c r="M34" s="3" t="inlineStr">
         <is>
           <t>Ausfuhr</t>
         </is>
       </c>
-      <c r="N34" s="9" t="inlineStr">
+      <c r="N34" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O34" s="9" t="inlineStr">
+      <c r="O34" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -3100,68 +3100,68 @@
           <t>Lager DE – WE Großbritannien (Ausfuhr, Post-Brexit)</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr"/>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H35" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J35" s="9" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K35" s="9" t="inlineStr">
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
       </c>
-      <c r="L35" s="10" t="inlineStr">
+      <c r="L35" s="4" t="inlineStr">
         <is>
           <t>G0</t>
         </is>
       </c>
-      <c r="M35" s="9" t="inlineStr">
+      <c r="M35" s="3" t="inlineStr">
         <is>
           <t>Ausfuhr</t>
         </is>
       </c>
-      <c r="N35" s="9" t="inlineStr">
+      <c r="N35" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O35" s="9" t="inlineStr">
+      <c r="O35" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -3174,75 +3174,75 @@
           <t>Strecke – Lieferant DE/EU – WE Großbritannien (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G36" s="9" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H36" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="I36" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J36" s="9" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K36" s="9" t="inlineStr">
+      <c r="K36" s="3" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
       </c>
-      <c r="L36" s="10" t="inlineStr">
+      <c r="L36" s="4" t="inlineStr">
         <is>
           <t>G0</t>
         </is>
       </c>
-      <c r="M36" s="9" t="inlineStr">
+      <c r="M36" s="3" t="inlineStr">
         <is>
           <t>Ausfuhr</t>
         </is>
       </c>
-      <c r="N36" s="9" t="inlineStr">
+      <c r="N36" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O36" s="9" t="inlineStr">
+      <c r="O36" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck)</t>
+          <t>Drittland-Ausfuhr über Heimat-UID (DE); KEIN Dreieck</t>
         </is>
       </c>
     </row>
@@ -3252,48 +3252,48 @@
           <t>Lager PL-Werk – WE Großbritannien (Ausfuhr) [Lücke: kein PL-Export-Stkz]</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>1702</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
           <t>PL5263841834</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H37" s="9" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="I37" s="9" t="inlineStr">
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>PL</t>
         </is>
       </c>
-      <c r="J37" s="9" t="inlineStr">
+      <c r="J37" s="3" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K37" s="9" t="inlineStr">
+      <c r="K37" s="3" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
@@ -3303,17 +3303,17 @@
           <t>⚠ kein SAP-Stkz (Treatment fehlt: export)</t>
         </is>
       </c>
-      <c r="M37" s="9" t="inlineStr">
+      <c r="M37" s="3" t="inlineStr">
         <is>
           <t>Ausfuhr</t>
         </is>
       </c>
-      <c r="N37" s="9" t="inlineStr">
+      <c r="N37" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O37" s="9" t="inlineStr">
+      <c r="O37" s="3" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -3326,22 +3326,22 @@
           <t>Strecke EXW – Lieferant Slowenien – WE Italien (SI ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -3351,47 +3351,47 @@
           <t>SI66423562</t>
         </is>
       </c>
-      <c r="G38" s="9" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H38" s="9" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="I38" s="9" t="inlineStr">
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="J38" s="9" t="inlineStr">
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K38" s="9" t="inlineStr">
+      <c r="K38" s="3" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L38" s="10" t="inlineStr">
+      <c r="L38" s="4" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="M38" s="9" t="inlineStr">
+      <c r="M38" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N38" s="9" t="inlineStr">
+      <c r="N38" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O38" s="9" t="inlineStr">
+      <c r="O38" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3404,22 +3404,22 @@
           <t>Strecke EXW – Lieferant Slowenien – WE Deutschland (SI ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -3429,47 +3429,47 @@
           <t>SI66423562</t>
         </is>
       </c>
-      <c r="G39" s="9" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H39" s="9" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="I39" s="9" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="J39" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="K39" s="9" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L39" s="10" t="inlineStr">
+      <c r="L39" s="4" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="M39" s="9" t="inlineStr">
+      <c r="M39" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N39" s="9" t="inlineStr">
+      <c r="N39" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O39" s="9" t="inlineStr">
+      <c r="O39" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3482,75 +3482,75 @@
           <t>Dreieck – Lieferant Frankreich → EPDE(DE) → WE Italien (Art. 141)</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E40" s="9" t="inlineStr"/>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G40" s="9" t="inlineStr">
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H40" s="9" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I40" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J40" s="9" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K40" s="9" t="inlineStr">
+      <c r="K40" s="3" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L40" s="10" t="inlineStr">
+      <c r="L40" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M40" s="9" t="inlineStr">
+      <c r="M40" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N40" s="9" t="inlineStr">
+      <c r="N40" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O40" s="9" t="inlineStr">
+      <c r="O40" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck)</t>
+          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck, Art. 141)</t>
         </is>
       </c>
     </row>
@@ -3560,75 +3560,75 @@
           <t>Dreieck – Lieferant Italien → EPDE(DE) → WE Spanien (Art. 141)</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>1701</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr"/>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>1701</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
           <t>DE449663039</t>
         </is>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS DE</t>
         </is>
       </c>
-      <c r="H41" s="9" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="I41" s="9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="J41" s="9" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="K41" s="9" t="inlineStr">
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>ESxxx</t>
         </is>
       </c>
-      <c r="L41" s="10" t="inlineStr">
+      <c r="L41" s="4" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M41" s="9" t="inlineStr">
+      <c r="M41" s="3" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
       </c>
-      <c r="N41" s="9" t="inlineStr">
+      <c r="N41" s="3" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="O41" s="9" t="inlineStr">
+      <c r="O41" s="3" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck)</t>
+          <t>Ship-to ohne EPDE-UID -&gt; BUKRS DE (Dreieck, Art. 141)</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3719,54 +3719,6 @@
       <c r="B6" s="8" t="inlineStr">
         <is>
           <t>WICHTIG: Diese Matrix bildet die SAP-Findung ab, die ship-to-/werks-/incoterm-basiert ist. Im EU-Reihengeschäft kann DIESELBE Länderkonstellation je nachdem, WER die Ware transportiert (Lieferant / mittlerer Unternehmer / Kunde) und an WELCHER Position der eigene Buchungskreis in der Kette steht (erster / mittlerer / letzter), eine ANDERE bewegte Lieferung und damit ein ANDERES Kennzeichen ergeben (EuGH C-245/04 EMAG; Art. 36a MwStSystRL / Quick Fixes). Die SAP-Findung modelliert diese Transportzuordnung nach aktuellem Stand NICHT explizit — sie leitet aus Werk/Ship-to/Incoterm ab. EXW ist der EINZIGE explizit abgebildete Transport-Trigger. Bei mehrgliedrigen Ketten mit abweichender Transportveranlassung daher gesondert prüfen: hier besteht zwischen der ship-to-basierten SAP-Logik und der transportbasierten Rechtslage eine bewusste Vereinfachung. Mit dem SAP-Team klären, ob die Findung Transportzuordnung überhaupt berücksichtigen soll.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>MIRO-Eingangsblatt</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Zweites Prinzip: die Eingangs-/Vorsteuerseite (MIRO). Blatt „MIRO_Eingang" leitet je Einkaufsfall das erwartete Eingangs-Kennzeichen ab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>MIRO — 4 Vorgänge</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>1) ig. Erwerb (eingehende Lieferung BEWEGT → Ankunftsland, Selbstveranlagung VE/VH/W5/EC/UR/BP/EP/LP/NP/IP, netto 0). 2) Inlandseinkauf (eingehende Lieferung RUHEND → Lieferant weist lokale MwSt aus, Vorsteuer VD/V2/B7/…). 3) Reverse Charge (DE §13b→DC, AT→RC, IT→VI). 4) Einfuhr Drittland (EUSt über EORI, kein Tabellen-MWSKZ). Sonderfall: eigene Ware ab Werk = kein Vorsteuervorgang (not relevant).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>MIRO — zwei Zusatz-Eingaben</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Anders als die Verkaufsseite braucht MIRO: (a) das LIEFERANTENLAND und (b) ob die EINGEHENDE Lieferung BEWEGT oder RUHEND ist. Genau das entscheidet zwischen ig. Erwerb (z. B. W5) und Inlandseinkauf (z. B. B7) — dieselbe Transportzuordnungs-Abhängigkeit wie oben.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>MIRO — offene Klärung</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Der Workshop hat MIRO als teils MANUELL markiert („steuerliches Abgangsland in der MIRO-Buchung korrekt pflegen"). Vor Automatisierung mit dem SAP-Team klären, ob die Findung MIRO automatisch ermitteln soll oder ob es ein manuell gepflegter Schritt bleibt.</t>
         </is>
       </c>
     </row>

</xml_diff>